<commit_message>
CHORE: Reviewed local papers
</commit_message>
<xml_diff>
--- a/RRL/Registry.xlsx
+++ b/RRL/Registry.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="145">
   <si>
     <t>Paper ID</t>
   </si>
@@ -454,6 +454,9 @@
   </si>
   <si>
     <t>Asi, G. M.; Anaya, K. O.; Piquero, J. R. M.; Romero, C. J. P.; Sales, Y. L. M.; Suñga, P. A. N.; Ibañez, M. M.; Ramos, R. I. A.</t>
+  </si>
+  <si>
+    <t>The non-significant correlations (r = -0.46 and 0.59, both p &gt; 0.05) demonstrate that self-reported capability is a weak proxy for actual financial discipline, supporting Odin's need for **behavioral profiling based on transaction data, not user surveys**.</t>
   </si>
 </sst>
 </file>
@@ -1081,7 +1084,8 @@
     <col min="4" max="4" width="20.5703125" style="3" customWidth="1"/>
     <col min="5" max="5" width="27.42578125" style="3" customWidth="1"/>
     <col min="6" max="6" width="20.5703125" style="3" customWidth="1"/>
-    <col min="7" max="9" width="13.7109375" style="3" customWidth="1"/>
+    <col min="7" max="8" width="13.7109375" style="3" customWidth="1"/>
+    <col min="9" max="9" width="50.7109375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1414,6 +1418,9 @@
       </c>
       <c r="F16" s="3" t="s">
         <v>46</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="89.25">

</xml_diff>

<commit_message>
CHORE: Summarized some papers
</commit_message>
<xml_diff>
--- a/RRL/Registry.xlsx
+++ b/RRL/Registry.xlsx
@@ -15,14 +15,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$B$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$B$41</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="160">
   <si>
     <t>Paper ID</t>
   </si>
@@ -457,6 +457,51 @@
   </si>
   <si>
     <t>The non-significant correlations (r = -0.46 and 0.59, both p &gt; 0.05) demonstrate that self-reported capability is a weak proxy for actual financial discipline, supporting Odin's need for **behavioral profiling based on transaction data, not user surveys**.</t>
+  </si>
+  <si>
+    <t>10.69569/jip.2025.063a</t>
+  </si>
+  <si>
+    <t>Espiritu, M. J.</t>
+  </si>
+  <si>
+    <t>Knowledge, Attitudes, and Practices in Financial Literacy among Business Administration Students in Urban College in the Philippines</t>
+  </si>
+  <si>
+    <t>10.47772/JIRISS.2025.91200252</t>
+  </si>
+  <si>
+    <t>Estorba, Vina L.; Relativo, John Lloyd C.; Relton, Stephanie Belle S.; Regis, Korina Jean M.</t>
+  </si>
+  <si>
+    <t>Ka-abag o Babag? Exploring the Lived Experiences in the Context of Financial Well-being of Microfinance Borrowers</t>
+  </si>
+  <si>
+    <t>Journal of Interdisciplinary Research and Innovations in Social Sciences</t>
+  </si>
+  <si>
+    <t>d3b07384-d9a0-4b6e-9c1a-5f8e2c7a4b6d</t>
+  </si>
+  <si>
+    <t>Flores, C. A. R.</t>
+  </si>
+  <si>
+    <t>Financial freedom of Filipinos in personal finance management</t>
+  </si>
+  <si>
+    <t>International Journal of the Humanities and Social Sciences</t>
+  </si>
+  <si>
+    <t>10.1145/3760557.3760578</t>
+  </si>
+  <si>
+    <t>Gabatin, R. A.; Sierra, S. M.; Maniago, M. G.; Capole, A.; Torres, R.</t>
+  </si>
+  <si>
+    <t>Understanding the Impulse Buying Behavior in the Digital Age: Influential Factors in Online Consumer Behavior</t>
+  </si>
+  <si>
+    <t>2025 16th International Conference on E-business, Management and Economics (ICEME)</t>
   </si>
 </sst>
 </file>
@@ -677,12 +722,6 @@
   </cellStyles>
   <dxfs count="17">
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -706,6 +745,12 @@
           <bgColor theme="7" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -792,14 +837,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:I37" totalsRowShown="0" headerRowDxfId="8" dataDxfId="9">
-  <autoFilter ref="A1:I37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:I41" totalsRowShown="0" headerRowDxfId="8" dataDxfId="9">
+  <autoFilter ref="A1:I41"/>
   <sortState ref="A2:I37">
     <sortCondition ref="B1:B37"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" name="Paper ID" dataDxfId="1"/>
-    <tableColumn id="2" name="Designation" dataDxfId="0"/>
+    <tableColumn id="1" name="Paper ID" dataDxfId="4"/>
+    <tableColumn id="2" name="Designation" dataDxfId="3"/>
     <tableColumn id="3" name="Year" dataDxfId="16"/>
     <tableColumn id="4" name="Authors" dataDxfId="15"/>
     <tableColumn id="5" name="Title" dataDxfId="14"/>
@@ -1075,15 +1120,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="13.7109375" style="3" customWidth="1"/>
     <col min="2" max="2" width="13.85546875" style="3" customWidth="1"/>
     <col min="3" max="3" width="13.7109375" style="3" customWidth="1"/>
     <col min="4" max="4" width="20.5703125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="27.42578125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="20.5703125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="30.7109375" style="3" customWidth="1"/>
+    <col min="6" max="6" width="25.7109375" style="3" customWidth="1"/>
     <col min="7" max="8" width="13.7109375" style="3" customWidth="1"/>
     <col min="9" max="9" width="50.7109375" style="3" customWidth="1"/>
   </cols>
@@ -1823,23 +1868,103 @@
         <v>139</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="102">
+    <row r="37" spans="1:6" ht="76.5">
       <c r="A37" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" s="3">
+        <v>2025</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="63.75">
+      <c r="A38" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C38" s="3">
+        <v>2026</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="38.25">
+      <c r="A39" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" s="3">
+        <v>2025</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="63.75">
+      <c r="A40" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C40" s="3">
+        <v>2025</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="102">
+      <c r="A41" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C37" s="3">
+      <c r="B41" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C41" s="3">
         <v>2024</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D41" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E41" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="F41" s="3" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1847,15 +1972,15 @@
   <sortState ref="A2:I36">
     <sortCondition ref="D1"/>
   </sortState>
-  <conditionalFormatting sqref="B2:B37">
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Algorithm-specific">
-      <formula>NOT(ISERROR(SEARCH("Algorithm-specific",B2)))</formula>
+  <conditionalFormatting sqref="B2:B41">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Local">
+      <formula>NOT(ISERROR(SEARCH("Local",B2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="International">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="International">
       <formula>NOT(ISERROR(SEARCH("International",B2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Local">
-      <formula>NOT(ISERROR(SEARCH("Local",B2)))</formula>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Algorithm-specific">
+      <formula>NOT(ISERROR(SEARCH("Algorithm-specific",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0" right="0" top="0.39370000000000011" bottom="0.39370000000000011" header="0" footer="0"/>

</xml_diff>

<commit_message>
CHORE: Tweaked summarizer skill; processed some papers
</commit_message>
<xml_diff>
--- a/RRL/Registry.xlsx
+++ b/RRL/Registry.xlsx
@@ -15,14 +15,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$B$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$B$43</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="212">
   <si>
     <t>Paper ID</t>
   </si>
@@ -649,6 +649,15 @@
   </si>
   <si>
     <t>"/budgeting-prevalence", "/budget-failure-points", "/cultural-obligations", "/fil-behavioral-patterns", "/fil-profile-construction", "/profile-dimensions", "/cultural-expense-types", "/fil-pfms-categories"</t>
+  </si>
+  <si>
+    <t>10.14744/sigma.2025.00119</t>
+  </si>
+  <si>
+    <t>Thankur, R. S.; Jadhav, A.</t>
+  </si>
+  <si>
+    <t>Expense tracker management system using machine learning</t>
   </si>
 </sst>
 </file>
@@ -900,21 +909,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Liberation Sans"/>
-        <scheme val="none"/>
-      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -945,6 +939,21 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Liberation Sans"/>
+        <scheme val="none"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -961,28 +970,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:I42" totalsRowShown="0" headerRowDxfId="3" dataDxfId="13">
-  <autoFilter ref="A1:I42">
-    <filterColumn colId="6">
-      <filters>
-        <filter val="2"/>
-        <filter val="2, 4, 5, 6, 7, 8, 12, 14, 15"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
-  <sortState ref="A5:I41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:I43" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="A1:I43"/>
+  <sortState ref="A2:I42">
     <sortCondition ref="B1:B42"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" name="Paper ID" dataDxfId="12"/>
-    <tableColumn id="2" name="Designation" dataDxfId="11"/>
-    <tableColumn id="3" name="Year" dataDxfId="10"/>
-    <tableColumn id="4" name="Authors" dataDxfId="9"/>
-    <tableColumn id="5" name="Title" dataDxfId="8"/>
-    <tableColumn id="6" name="Venue" dataDxfId="7"/>
-    <tableColumn id="7" name="Topics" dataDxfId="6"/>
-    <tableColumn id="8" name="Tags" dataDxfId="5"/>
-    <tableColumn id="9" name="Notes" dataDxfId="4"/>
+    <tableColumn id="1" name="Paper ID" dataDxfId="11"/>
+    <tableColumn id="2" name="Designation" dataDxfId="10"/>
+    <tableColumn id="3" name="Year" dataDxfId="9"/>
+    <tableColumn id="4" name="Authors" dataDxfId="8"/>
+    <tableColumn id="5" name="Title" dataDxfId="7"/>
+    <tableColumn id="6" name="Venue" dataDxfId="6"/>
+    <tableColumn id="7" name="Topics" dataDxfId="5"/>
+    <tableColumn id="8" name="Tags" dataDxfId="4"/>
+    <tableColumn id="9" name="Notes" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1251,7 +1253,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="4" width="25.7109375" style="2" customWidth="1"/>
@@ -1316,52 +1318,49 @@
         <v>165</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="99.95" hidden="1" customHeight="1">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C4" s="1">
         <v>2025</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" ht="99.95" hidden="1" customHeight="1">
-      <c r="A4" s="2" t="s">
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A5" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="2">
-        <v>2026</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="99.95" hidden="1" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>10</v>
@@ -1370,174 +1369,168 @@
         <v>2026</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="99.95" hidden="1" customHeight="1">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="99.95" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="2">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="99.95" hidden="1" customHeight="1">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="99.95" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>120</v>
+        <v>54</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>121</v>
+        <v>55</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>122</v>
+        <v>56</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>123</v>
+        <v>57</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="99.95" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C8" s="2">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="G8" s="2">
-        <v>2</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="99.95" hidden="1" customHeight="1">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="99.95" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>74</v>
+        <v>124</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C9" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="G9" s="2">
+        <v>2</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="2">
         <v>2025</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="99.95" hidden="1" customHeight="1">
-      <c r="A10" s="2" t="s">
+    <row r="11" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="2">
+      <c r="B11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="2">
         <v>2024</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="99.95" hidden="1" customHeight="1">
-      <c r="A11" s="2" t="s">
+    <row r="12" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A12" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="2">
-        <v>2025</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="99.95" hidden="1" customHeight="1">
-      <c r="A12" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>15</v>
@@ -1546,50 +1539,50 @@
         <v>2025</v>
       </c>
       <c r="D12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G13" s="2">
         <v>1</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H13" s="2" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="99.95" hidden="1" customHeight="1">
-      <c r="A13" s="2" t="s">
+    <row r="14" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A14" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="2">
-        <v>2026</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="99.95" hidden="1" customHeight="1">
-      <c r="A14" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>15</v>
@@ -1598,79 +1591,79 @@
         <v>2026</v>
       </c>
       <c r="D14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="99.95" hidden="1" customHeight="1">
-      <c r="A15" s="2" t="s">
+    <row r="16" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A16" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="2">
+      <c r="B16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="2">
         <v>2025</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F16" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H16" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="I16" s="2" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="99.95" hidden="1" customHeight="1">
-      <c r="A16" s="2" t="s">
+    <row r="17" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A17" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A17" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>15</v>
@@ -1679,313 +1672,313 @@
         <v>2024</v>
       </c>
       <c r="D17" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="G18" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="H18" s="2" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A18" s="2" t="s">
+    <row r="19" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A19" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C18" s="2">
+      <c r="B19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="2">
         <v>2026</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G18" s="2">
-        <v>1</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A19" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C19" s="2">
-        <v>2021</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>72</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G19" s="2" t="s">
-        <v>189</v>
+      <c r="G19" s="2">
+        <v>1</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="99.95" hidden="1" customHeight="1">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="99.95" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C20" s="2">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" ht="99.95" hidden="1" customHeight="1">
+      <c r="G20" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="99.95" customHeight="1">
       <c r="A21" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A22" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="2">
+      <c r="B22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="2">
         <v>2025</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F22" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="H22" s="2" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A22" s="2" t="s">
+    <row r="23" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A23" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="2">
+      <c r="B23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="2">
         <v>2024</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="G23" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="H23" s="2" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A23" s="2" t="s">
+    <row r="24" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A24" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C23" s="2">
+      <c r="B24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="2">
         <v>2025</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E24" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="G24" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="H23" s="2" t="s">
+      <c r="H24" s="2" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A24" s="2" t="s">
+    <row r="25" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A25" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C24" s="2">
+      <c r="B25" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="2">
         <v>2024</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D25" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E25" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F25" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="G25" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="H24" s="2" t="s">
+      <c r="H25" s="2" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A25" s="2" t="s">
+    <row r="26" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A26" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C25" s="2">
+      <c r="B26" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="2">
         <v>2025</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E26" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="H25" s="2" t="s">
+      <c r="H26" s="2" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A26" s="2" t="s">
+    <row r="27" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A27" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" s="2">
+      <c r="B27" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C27" s="2">
         <v>2024</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E27" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F27" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A27" s="2" t="s">
+    <row r="28" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A28" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C27" s="2">
+      <c r="B28" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28" s="2">
         <v>2025</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E28" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="F28" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="G28" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="H28" s="2" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A28" s="2" t="s">
+    <row r="29" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A29" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C28" s="2">
+      <c r="B29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29" s="2">
         <v>2024</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D29" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E29" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="F29" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A29" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C29" s="2">
-        <v>2025</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>106</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>180</v>
@@ -1994,9 +1987,9 @@
         <v>199</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="99.95" hidden="1" customHeight="1">
+    <row r="30" spans="1:8" ht="99.95" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>15</v>
@@ -2005,48 +1998,48 @@
         <v>2025</v>
       </c>
       <c r="D30" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C31" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E31" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="F31" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="G30" s="2">
+      <c r="G31" s="2">
         <v>1</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="H31" s="2" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A31" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C31" s="2">
-        <v>2023</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="99.95" hidden="1" customHeight="1">
+    <row r="32" spans="1:8" ht="99.95" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>74</v>
       </c>
@@ -2054,53 +2047,53 @@
         <v>15</v>
       </c>
       <c r="C32" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" s="2">
         <v>2024</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D33" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E33" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="F33" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="G33" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="H33" s="2" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A33" s="2" t="s">
+    <row r="34" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A34" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C33" s="2">
-        <v>2025</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A34" s="2" t="s">
-        <v>128</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>15</v>
@@ -2109,142 +2102,142 @@
         <v>2025</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C35" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="E35" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="F35" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="G35" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="H34" s="2" t="s">
+      <c r="H35" s="2" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A35" s="2" t="s">
+    <row r="36" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A36" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C35" s="2">
+      <c r="B36" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36" s="2">
         <v>2026</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="D36" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="E36" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="F36" s="2" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A36" s="2" t="s">
+    <row r="37" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A37" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C36" s="2">
+      <c r="B37" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" s="2">
         <v>2023</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="D37" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E37" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="F37" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A37" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C37" s="2">
-        <v>2025</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>180</v>
       </c>
       <c r="H37" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C38" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="H38" s="2" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A38" s="2" t="s">
+    <row r="39" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A39" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C38" s="2">
+      <c r="B39" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" s="2">
         <v>2026</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="D39" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="E39" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="F39" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A39" s="2" t="s">
+    <row r="40" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A40" s="2" t="s">
         <v>152</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C39" s="2">
-        <v>2025</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A40" s="2" t="s">
-        <v>156</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>15</v>
@@ -2253,24 +2246,24 @@
         <v>2025</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="G40" s="2">
-        <v>1</v>
+        <v>155</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>180</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="99.95" hidden="1" customHeight="1">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="99.95" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>15</v>
@@ -2279,38 +2272,64 @@
         <v>2025</v>
       </c>
       <c r="D41" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="G41" s="2">
+        <v>1</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C42" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E42" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="F41" s="2" t="s">
+      <c r="F42" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G41" s="2" t="s">
+      <c r="G42" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="H41" s="2" t="s">
+      <c r="H42" s="2" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="99.95" hidden="1" customHeight="1">
-      <c r="A42" s="2" t="s">
+    <row r="43" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A43" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C42" s="2">
+      <c r="B43" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C43" s="2">
         <v>2024</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="D43" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E42" s="2" t="s">
+      <c r="E43" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="F42" s="2" t="s">
+      <c r="F43" s="2" t="s">
         <v>72</v>
       </c>
     </row>
@@ -2318,7 +2337,7 @@
   <sortState ref="A2:I36">
     <sortCondition ref="D1"/>
   </sortState>
-  <conditionalFormatting sqref="B2:B42">
+  <conditionalFormatting sqref="B2:B43">
     <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Local">
       <formula>NOT(ISERROR(SEARCH("Local",B2)))</formula>
     </cfRule>

</xml_diff>

<commit_message>
CHORE: Deprecated Registry; migrated to Scribbr
Modified several file locations; fixed details of some files
</commit_message>
<xml_diff>
--- a/RRL/Registry.xlsx
+++ b/RRL/Registry.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$B$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$B$44</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -234,9 +234,6 @@
     <t>AI-Based Wealth Advisory System using Machine Learning and Predictive Analytics for Personalized Budget Planning</t>
   </si>
   <si>
-    <t>International Journal of Advanced Research in Computer Science and Technology</t>
-  </si>
-  <si>
     <t>f7d9e3a2-5b1c-4e8a-9d2f-6b4e8c7a3d1f</t>
   </si>
   <si>
@@ -513,24 +510,9 @@
     <t>Financial Literacy and Financial Health of Public Junior High School Teachers</t>
   </si>
   <si>
-    <t>2, 4, 5, 6, 7, 8, 12, 14, 15</t>
-  </si>
-  <si>
     <t>1, 10</t>
   </si>
   <si>
-    <t>"/pfms-limitations", "/pfms-gap", "/budget-rec-algorithms", "/forecasting-methods", "/lstm-spending-applied", "/anomaly-approaches", "/alert-design", "/isolation-forest", "/security-standards", "/privacy-by-design", "/budget-alloc-algos", "/eval-pfms-applied", "/sus"</t>
-  </si>
-  <si>
-    <t>"/intelligent-vs-literacy", "/profile-dimensions"</t>
-  </si>
-  <si>
-    <t>1, 4, 5, 10</t>
-  </si>
-  <si>
-    <t>"/expenditure-patterns", "/budgeting-prevalence", "/intelligent-vs-literacy", "/strategy-mechanics", "/budget-rec-formulation", "/western-taxonomy-gap", "/fil-behavioral-patterns"</t>
-  </si>
-  <si>
     <t>"/pfms-limitations", "/pfms-gap"</t>
   </si>
   <si>
@@ -658,6 +640,24 @@
   </si>
   <si>
     <t>Expense tracker management system using machine learning</t>
+  </si>
+  <si>
+    <t>International Journal of Advanced Research in Computer Science &amp; Technology</t>
+  </si>
+  <si>
+    <t>Sigma Journal of Engineering and Natural Sciences</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.14236/ewic/BCSHCI2023.1 </t>
+  </si>
+  <si>
+    <t>Alenazi, M.; Sas, C.</t>
+  </si>
+  <si>
+    <t>Evaluating budgeting apps: Limited support for budgeting compared to tracking</t>
+  </si>
+  <si>
+    <t>Electronic Workshops in Computing</t>
   </si>
 </sst>
 </file>
@@ -970,8 +970,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:I43" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="A1:I43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:I44" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="A1:I44"/>
   <sortState ref="A2:I42">
     <sortCondition ref="B1:B42"/>
   </sortState>
@@ -1253,7 +1253,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="4" width="25.7109375" style="2" customWidth="1"/>
@@ -1309,18 +1309,12 @@
         <v>69</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>165</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="99.95" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>67</v>
@@ -1329,10 +1323,13 @@
         <v>2025</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="99.95" customHeight="1">
@@ -1359,204 +1356,189 @@
       <c r="I4" s="1"/>
     </row>
     <row r="5" spans="1:9" ht="99.95" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="A5" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="2">
-        <v>2026</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>38</v>
-      </c>
+      <c r="C5" s="1">
+        <v>2023</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
     </row>
     <row r="6" spans="1:9" ht="99.95" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>166</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="99.95" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="2">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>168</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="99.95" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>120</v>
+        <v>54</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C8" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>121</v>
+        <v>55</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>122</v>
+        <v>56</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>123</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="99.95" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C9" s="2">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="G9" s="2">
-        <v>2</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>169</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="99.95" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="2">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>141</v>
+        <v>124</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>170</v>
+        <v>126</v>
+      </c>
+      <c r="G10" s="2">
+        <v>2</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="99.95" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>14</v>
+        <v>73</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C11" s="2">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>16</v>
+        <v>140</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>17</v>
+        <v>139</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>18</v>
+        <v>141</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="99.95" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C12" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="99.95" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>15</v>
@@ -1565,50 +1547,50 @@
         <v>2025</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G13" s="2">
-        <v>1</v>
+        <v>22</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>168</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="99.95" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C14" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>179</v>
+        <v>30</v>
+      </c>
+      <c r="G14" s="2">
+        <v>1</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="99.95" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>15</v>
@@ -1617,79 +1599,79 @@
         <v>2026</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="99.95" customHeight="1">
       <c r="A16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A17" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="2">
+      <c r="B17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="2">
         <v>2025</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A17" s="2" t="s">
+      <c r="G17" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A18" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A18" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>15</v>
@@ -1698,324 +1680,324 @@
         <v>2024</v>
       </c>
       <c r="D18" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="G19" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G20" s="2">
+        <v>1</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="2">
+        <v>2021</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="H24" s="2" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A19" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C19" s="2">
-        <v>2026</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G19" s="2">
-        <v>1</v>
-      </c>
-      <c r="H19" s="2" t="s">
+    <row r="25" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="H25" s="2" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A20" s="2" t="s">
+    <row r="26" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" s="2">
-        <v>2021</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A21" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A22" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="2">
-        <v>2025</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A23" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C23" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A24" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C24" s="2">
-        <v>2025</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A25" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C25" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A26" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" s="2">
-        <v>2025</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>174</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="99.95" customHeight="1">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="99.95" customHeight="1">
       <c r="A27" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C27" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A28" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C27" s="2">
+      <c r="B28" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28" s="2">
         <v>2024</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E28" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="F28" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A28" s="2" t="s">
+    <row r="29" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C28" s="2">
-        <v>2025</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="E29" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="F29" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A30" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="F28" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A29" s="2" t="s">
+      <c r="B30" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C30" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C29" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D29" s="2" t="s">
+      <c r="E30" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="F30" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="G30" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A31" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A30" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C30" s="2">
-        <v>2025</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A31" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>15</v>
@@ -2024,102 +2006,102 @@
         <v>2025</v>
       </c>
       <c r="D31" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="99.95" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C32" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="F32" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F31" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="G31" s="2">
+      <c r="G32" s="2">
         <v>1</v>
       </c>
-      <c r="H31" s="2" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="99.95" customHeight="1">
-      <c r="A32" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C32" s="2">
-        <v>2023</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>180</v>
-      </c>
       <c r="H32" s="2" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="99.95" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C33" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="99.95" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>117</v>
+        <v>73</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C34" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>198</v>
+        <v>173</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="99.95" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>15</v>
@@ -2128,142 +2110,142 @@
         <v>2025</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="99.95" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C36" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>135</v>
+        <v>130</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="99.95" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C37" s="2">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>199</v>
+        <v>134</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="99.95" customHeight="1">
       <c r="A38" s="2" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C38" s="2">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>26</v>
+        <v>138</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="99.95" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C39" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>151</v>
+        <v>26</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="99.95" customHeight="1">
       <c r="A40" s="2" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C40" s="2">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>206</v>
+        <v>150</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="99.95" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>15</v>
@@ -2272,24 +2254,24 @@
         <v>2025</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="G41" s="2">
-        <v>1</v>
+        <v>154</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>174</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="99.95" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>15</v>
@@ -2298,46 +2280,72 @@
         <v>2025</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>189</v>
+        <v>158</v>
+      </c>
+      <c r="G42" s="2">
+        <v>1</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="99.95" customHeight="1">
       <c r="A43" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C43" s="2">
+        <v>2025</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="99.95" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C44" s="2">
+        <v>2024</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B43" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C43" s="2">
-        <v>2024</v>
-      </c>
-      <c r="D43" s="2" t="s">
+      <c r="E44" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E43" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>72</v>
+      <c r="F44" s="2" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
   <sortState ref="A2:I36">
     <sortCondition ref="D1"/>
   </sortState>
-  <conditionalFormatting sqref="B2:B43">
+  <conditionalFormatting sqref="B2:B44">
     <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Local">
       <formula>NOT(ISERROR(SEARCH("Local",B2)))</formula>
     </cfRule>

</xml_diff>